<commit_message>
application with multiple collateral ids handled
</commit_message>
<xml_diff>
--- a/Dummy input data/Dummy CKYC/CKYC.xlsx
+++ b/Dummy input data/Dummy CKYC/CKYC.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X89"/>
+  <dimension ref="A1:X95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9629,6 +9629,656 @@
         <v>5000980</v>
       </c>
       <c r="X89" t="inlineStr">
+        <is>
+          <t>15-MAY-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>16-09-2026</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Thane</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>16-SEP-26</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>APPL00090030</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>ARGFLLAPMUM2000000903001</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>VINOD RAMCHANDRA SAWANT</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>GLBCUST00000090301</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>14-JUL-72</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>VINOD</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>RAMCHANDRA</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>SAWANT</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>AXSPS3031K</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>+91--9800090301</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>vinod.sawant72@gmail.com</t>
+        </is>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>Flat No. 802, 8th Floor, Neelkanth Heights, Pokharan Road No. 2, Thane West, Thane, Maharashtra- 400610, India</t>
+        </is>
+      </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>Low Risk</t>
+        </is>
+      </c>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W90" t="n">
+        <v>5000980</v>
+      </c>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>15-MAY-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>16-09-2026</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Thane</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>16-SEP-26</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>APPL00090030</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>ARGFLLAPMUM2000000903001</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Co-Applicant</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>MEGHA VINOD SAWANT</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>GLBCUST00000090302</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>22-MAR-76</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>MEGHA</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>VINOD</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>SAWANT</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>BYSPS3032L</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>+91--9800090302</t>
+        </is>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>Flat No. 802, 8th Floor, Neelkanth Heights, Pokharan Road No. 2, Thane West, Thane, Maharashtra- 400610, India</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>Low Risk</t>
+        </is>
+      </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W91" t="n">
+        <v>5000980</v>
+      </c>
+      <c r="X91" t="inlineStr">
+        <is>
+          <t>15-MAY-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>16-09-2026</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Thane</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>16-SEP-26</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>APPL00090030</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>ARGFLLAPMUM2000000903001</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Co-Applicant</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>non_individual</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>SAWANT ELECTRICALS</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Sole Proprietorship Firm</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>GLBCUST00000090303</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>01-APR-05</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>AXSPS3031K</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>+91--9900090303</t>
+        </is>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>Shop No. 6, Ground Floor, Gokul Arcade, Station Road, Naupada, Thane West, Thane, Maharashtra- 400601, India</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>Low Risk</t>
+        </is>
+      </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W92" t="n">
+        <v>5000980</v>
+      </c>
+      <c r="X92" t="inlineStr">
+        <is>
+          <t>15-MAY-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>16-09-2026</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Thane</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>16-SEP-26</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>APPL00090030</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>ARGFLLAPMUM2000000903001</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Co-Applicant</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>RAMCHANDRA GANPAT SAWANT</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>GLBCUST00000090304</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>03-JAN-48</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>RAMCHANDRA</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>GANPAT</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>SAWANT</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>ACSPS3034M</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>+91--9800090304</t>
+        </is>
+      </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>Flat No. 802, 8th Floor, Neelkanth Heights, Pokharan Road No. 2, Thane West, Thane, Maharashtra- 400610, India</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>Low Risk</t>
+        </is>
+      </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W93" t="n">
+        <v>5000980</v>
+      </c>
+      <c r="X93" t="inlineStr">
+        <is>
+          <t>15-MAY-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>08-09-2026</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>08-SEP-26</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>APPL00090031</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>ARGFLLAPMUM2000000903101</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>ASHOK BHIKAJI KULKARNI</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>GLBCUST00000090311</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>19-FEB-70</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>ASHOK</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>BHIKAJI</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>KULKARNI</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>ALKPK3111N</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>+91--9800090311</t>
+        </is>
+      </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>Flat No. 101, Sai Krupa Apartment, Karve Nagar, Pune, Maharashtra- 411052, India</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>Low Risk</t>
+        </is>
+      </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W94" t="n">
+        <v>5000980</v>
+      </c>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>15-MAY-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>08-09-2026</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>08-SEP-26</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>APPL00090031</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>ARGFLLAPMUM2000000903101</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Co-Applicant</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>SEEMA ASHOK KULKARNI</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>GLBCUST00000090312</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>07-AUG-74</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>SEEMA</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>ASHOK</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>KULKARNI</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>BMKPK3112P</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>+91--9800090312</t>
+        </is>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>Flat No. 101, Sai Krupa Apartment, Karve Nagar, Pune, Maharashtra- 411052, India</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>Low Risk</t>
+        </is>
+      </c>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W95" t="n">
+        <v>5000980</v>
+      </c>
+      <c r="X95" t="inlineStr">
         <is>
           <t>15-MAY-26</t>
         </is>

</xml_diff>